<commit_message>
chore: update WordCountData.xlsx with latest recorded entries
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/WordCountData.xlsx
+++ b/WordCountData.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E139"/>
+  <dimension ref="A1:E230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2502,7 +2502,7 @@
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
-        <v>45906.84478628391</v>
+        <v>45906.84478628472</v>
       </c>
       <c r="B139" t="n">
         <v>549</v>
@@ -2515,6 +2515,1553 @@
       </c>
       <c r="E139" t="n">
         <v>8.47580494456402</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B140" t="n">
+        <v>113</v>
+      </c>
+      <c r="C140" t="n">
+        <v>297</v>
+      </c>
+      <c r="D140" t="n">
+        <v>22.91783614707553</v>
+      </c>
+      <c r="E140" t="n">
+        <v>22.91783614707553</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B141" t="n">
+        <v>211</v>
+      </c>
+      <c r="C141" t="n">
+        <v>597</v>
+      </c>
+      <c r="D141" t="n">
+        <v>29.29897897578328</v>
+      </c>
+      <c r="E141" t="n">
+        <v>29.29897897578328</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B142" t="n">
+        <v>211</v>
+      </c>
+      <c r="C142" t="n">
+        <v>897</v>
+      </c>
+      <c r="D142" t="n">
+        <v>29.29897897578328</v>
+      </c>
+      <c r="E142" t="n">
+        <v>29.29897897578328</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B143" t="n">
+        <v>211</v>
+      </c>
+      <c r="C143" t="n">
+        <v>1197</v>
+      </c>
+      <c r="D143" t="n">
+        <v>29.29897897578328</v>
+      </c>
+      <c r="E143" t="n">
+        <v>29.29897897578328</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B144" t="n">
+        <v>268</v>
+      </c>
+      <c r="C144" t="n">
+        <v>1497</v>
+      </c>
+      <c r="D144" t="n">
+        <v>11.01239930853471</v>
+      </c>
+      <c r="E144" t="n">
+        <v>11.01239930853471</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B145" t="n">
+        <v>277</v>
+      </c>
+      <c r="C145" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D145" t="n">
+        <v>9.247434217234732</v>
+      </c>
+      <c r="E145" t="n">
+        <v>9.247434217234732</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B146" t="n">
+        <v>477</v>
+      </c>
+      <c r="C146" t="n">
+        <v>2097</v>
+      </c>
+      <c r="D146" t="n">
+        <v>13.65461330578994</v>
+      </c>
+      <c r="E146" t="n">
+        <v>13.65461330578994</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B147" t="n">
+        <v>498</v>
+      </c>
+      <c r="C147" t="n">
+        <v>2397</v>
+      </c>
+      <c r="D147" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E147" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B148" t="n">
+        <v>498</v>
+      </c>
+      <c r="C148" t="n">
+        <v>2697</v>
+      </c>
+      <c r="D148" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E148" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B149" t="n">
+        <v>498</v>
+      </c>
+      <c r="C149" t="n">
+        <v>2997</v>
+      </c>
+      <c r="D149" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E149" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B150" t="n">
+        <v>498</v>
+      </c>
+      <c r="C150" t="n">
+        <v>3297</v>
+      </c>
+      <c r="D150" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E150" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B151" t="n">
+        <v>498</v>
+      </c>
+      <c r="C151" t="n">
+        <v>3597</v>
+      </c>
+      <c r="D151" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E151" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B152" t="n">
+        <v>498</v>
+      </c>
+      <c r="C152" t="n">
+        <v>3897</v>
+      </c>
+      <c r="D152" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E152" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B153" t="n">
+        <v>498</v>
+      </c>
+      <c r="C153" t="n">
+        <v>4198</v>
+      </c>
+      <c r="D153" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E153" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B154" t="n">
+        <v>498</v>
+      </c>
+      <c r="C154" t="n">
+        <v>4498</v>
+      </c>
+      <c r="D154" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E154" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B155" t="n">
+        <v>498</v>
+      </c>
+      <c r="C155" t="n">
+        <v>4798</v>
+      </c>
+      <c r="D155" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E155" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B156" t="n">
+        <v>498</v>
+      </c>
+      <c r="C156" t="n">
+        <v>5098</v>
+      </c>
+      <c r="D156" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E156" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B157" t="n">
+        <v>498</v>
+      </c>
+      <c r="C157" t="n">
+        <v>5398</v>
+      </c>
+      <c r="D157" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E157" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B158" t="n">
+        <v>498</v>
+      </c>
+      <c r="C158" t="n">
+        <v>5698</v>
+      </c>
+      <c r="D158" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E158" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B159" t="n">
+        <v>498</v>
+      </c>
+      <c r="C159" t="n">
+        <v>5998</v>
+      </c>
+      <c r="D159" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E159" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B160" t="n">
+        <v>498</v>
+      </c>
+      <c r="C160" t="n">
+        <v>6298</v>
+      </c>
+      <c r="D160" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E160" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B161" t="n">
+        <v>498</v>
+      </c>
+      <c r="C161" t="n">
+        <v>6598</v>
+      </c>
+      <c r="D161" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E161" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B162" t="n">
+        <v>498</v>
+      </c>
+      <c r="C162" t="n">
+        <v>6898</v>
+      </c>
+      <c r="D162" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E162" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B163" t="n">
+        <v>498</v>
+      </c>
+      <c r="C163" t="n">
+        <v>7198</v>
+      </c>
+      <c r="D163" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E163" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B164" t="n">
+        <v>498</v>
+      </c>
+      <c r="C164" t="n">
+        <v>7498</v>
+      </c>
+      <c r="D164" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E164" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B165" t="n">
+        <v>498</v>
+      </c>
+      <c r="C165" t="n">
+        <v>7799</v>
+      </c>
+      <c r="D165" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E165" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B166" t="n">
+        <v>498</v>
+      </c>
+      <c r="C166" t="n">
+        <v>8099</v>
+      </c>
+      <c r="D166" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E166" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B167" t="n">
+        <v>498</v>
+      </c>
+      <c r="C167" t="n">
+        <v>8399</v>
+      </c>
+      <c r="D167" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E167" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B168" t="n">
+        <v>498</v>
+      </c>
+      <c r="C168" t="n">
+        <v>8699</v>
+      </c>
+      <c r="D168" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E168" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B169" t="n">
+        <v>498</v>
+      </c>
+      <c r="C169" t="n">
+        <v>8999</v>
+      </c>
+      <c r="D169" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E169" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B170" t="n">
+        <v>498</v>
+      </c>
+      <c r="C170" t="n">
+        <v>9299</v>
+      </c>
+      <c r="D170" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E170" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B171" t="n">
+        <v>498</v>
+      </c>
+      <c r="C171" t="n">
+        <v>9599</v>
+      </c>
+      <c r="D171" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E171" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B172" t="n">
+        <v>498</v>
+      </c>
+      <c r="C172" t="n">
+        <v>9899</v>
+      </c>
+      <c r="D172" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E172" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B173" t="n">
+        <v>498</v>
+      </c>
+      <c r="C173" t="n">
+        <v>10199</v>
+      </c>
+      <c r="D173" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E173" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B174" t="n">
+        <v>498</v>
+      </c>
+      <c r="C174" t="n">
+        <v>10499</v>
+      </c>
+      <c r="D174" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E174" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B175" t="n">
+        <v>498</v>
+      </c>
+      <c r="C175" t="n">
+        <v>10799</v>
+      </c>
+      <c r="D175" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E175" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B176" t="n">
+        <v>498</v>
+      </c>
+      <c r="C176" t="n">
+        <v>11099</v>
+      </c>
+      <c r="D176" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E176" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B177" t="n">
+        <v>498</v>
+      </c>
+      <c r="C177" t="n">
+        <v>11399</v>
+      </c>
+      <c r="D177" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E177" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B178" t="n">
+        <v>498</v>
+      </c>
+      <c r="C178" t="n">
+        <v>11700</v>
+      </c>
+      <c r="D178" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E178" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B179" t="n">
+        <v>498</v>
+      </c>
+      <c r="C179" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D179" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E179" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B180" t="n">
+        <v>498</v>
+      </c>
+      <c r="C180" t="n">
+        <v>12300</v>
+      </c>
+      <c r="D180" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E180" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B181" t="n">
+        <v>498</v>
+      </c>
+      <c r="C181" t="n">
+        <v>12600</v>
+      </c>
+      <c r="D181" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E181" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B182" t="n">
+        <v>498</v>
+      </c>
+      <c r="C182" t="n">
+        <v>12900</v>
+      </c>
+      <c r="D182" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E182" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B183" t="n">
+        <v>498</v>
+      </c>
+      <c r="C183" t="n">
+        <v>13200</v>
+      </c>
+      <c r="D183" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E183" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B184" t="n">
+        <v>498</v>
+      </c>
+      <c r="C184" t="n">
+        <v>13500</v>
+      </c>
+      <c r="D184" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E184" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B185" t="n">
+        <v>498</v>
+      </c>
+      <c r="C185" t="n">
+        <v>13800</v>
+      </c>
+      <c r="D185" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E185" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B186" t="n">
+        <v>498</v>
+      </c>
+      <c r="C186" t="n">
+        <v>14100</v>
+      </c>
+      <c r="D186" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E186" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B187" t="n">
+        <v>498</v>
+      </c>
+      <c r="C187" t="n">
+        <v>14400</v>
+      </c>
+      <c r="D187" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E187" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B188" t="n">
+        <v>498</v>
+      </c>
+      <c r="C188" t="n">
+        <v>14700</v>
+      </c>
+      <c r="D188" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E188" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B189" t="n">
+        <v>498</v>
+      </c>
+      <c r="C189" t="n">
+        <v>15001</v>
+      </c>
+      <c r="D189" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E189" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B190" t="n">
+        <v>498</v>
+      </c>
+      <c r="C190" t="n">
+        <v>15301</v>
+      </c>
+      <c r="D190" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E190" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B191" t="n">
+        <v>498</v>
+      </c>
+      <c r="C191" t="n">
+        <v>15601</v>
+      </c>
+      <c r="D191" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E191" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B192" t="n">
+        <v>498</v>
+      </c>
+      <c r="C192" t="n">
+        <v>15901</v>
+      </c>
+      <c r="D192" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E192" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B193" t="n">
+        <v>498</v>
+      </c>
+      <c r="C193" t="n">
+        <v>16201</v>
+      </c>
+      <c r="D193" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E193" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B194" t="n">
+        <v>498</v>
+      </c>
+      <c r="C194" t="n">
+        <v>16501</v>
+      </c>
+      <c r="D194" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E194" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B195" t="n">
+        <v>498</v>
+      </c>
+      <c r="C195" t="n">
+        <v>16801</v>
+      </c>
+      <c r="D195" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E195" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B196" t="n">
+        <v>498</v>
+      </c>
+      <c r="C196" t="n">
+        <v>17101</v>
+      </c>
+      <c r="D196" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E196" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B197" t="n">
+        <v>498</v>
+      </c>
+      <c r="C197" t="n">
+        <v>17401</v>
+      </c>
+      <c r="D197" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E197" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B198" t="n">
+        <v>498</v>
+      </c>
+      <c r="C198" t="n">
+        <v>17701</v>
+      </c>
+      <c r="D198" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E198" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B199" t="n">
+        <v>498</v>
+      </c>
+      <c r="C199" t="n">
+        <v>18001</v>
+      </c>
+      <c r="D199" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E199" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B200" t="n">
+        <v>498</v>
+      </c>
+      <c r="C200" t="n">
+        <v>18301</v>
+      </c>
+      <c r="D200" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E200" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B201" t="n">
+        <v>498</v>
+      </c>
+      <c r="C201" t="n">
+        <v>18602</v>
+      </c>
+      <c r="D201" t="n">
+        <v>14.07996070958818</v>
+      </c>
+      <c r="E201" t="n">
+        <v>14.07996070958818</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B202" t="n">
+        <v>499</v>
+      </c>
+      <c r="C202" t="n">
+        <v>18902</v>
+      </c>
+      <c r="D202" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E202" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B203" t="n">
+        <v>499</v>
+      </c>
+      <c r="C203" t="n">
+        <v>19202</v>
+      </c>
+      <c r="D203" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E203" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B204" t="n">
+        <v>499</v>
+      </c>
+      <c r="C204" t="n">
+        <v>19502</v>
+      </c>
+      <c r="D204" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E204" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B205" t="n">
+        <v>499</v>
+      </c>
+      <c r="C205" t="n">
+        <v>19802</v>
+      </c>
+      <c r="D205" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E205" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B206" t="n">
+        <v>499</v>
+      </c>
+      <c r="C206" t="n">
+        <v>20102</v>
+      </c>
+      <c r="D206" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E206" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B207" t="n">
+        <v>499</v>
+      </c>
+      <c r="C207" t="n">
+        <v>20402</v>
+      </c>
+      <c r="D207" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E207" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B208" t="n">
+        <v>499</v>
+      </c>
+      <c r="C208" t="n">
+        <v>20702</v>
+      </c>
+      <c r="D208" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E208" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B209" t="n">
+        <v>499</v>
+      </c>
+      <c r="C209" t="n">
+        <v>21002</v>
+      </c>
+      <c r="D209" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E209" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B210" t="n">
+        <v>499</v>
+      </c>
+      <c r="C210" t="n">
+        <v>21302</v>
+      </c>
+      <c r="D210" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E210" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B211" t="n">
+        <v>499</v>
+      </c>
+      <c r="C211" t="n">
+        <v>21602</v>
+      </c>
+      <c r="D211" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E211" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B212" t="n">
+        <v>499</v>
+      </c>
+      <c r="C212" t="n">
+        <v>21903</v>
+      </c>
+      <c r="D212" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E212" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B213" t="n">
+        <v>499</v>
+      </c>
+      <c r="C213" t="n">
+        <v>22203</v>
+      </c>
+      <c r="D213" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E213" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B214" t="n">
+        <v>499</v>
+      </c>
+      <c r="C214" t="n">
+        <v>22503</v>
+      </c>
+      <c r="D214" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E214" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B215" t="n">
+        <v>499</v>
+      </c>
+      <c r="C215" t="n">
+        <v>22803</v>
+      </c>
+      <c r="D215" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E215" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B216" t="n">
+        <v>499</v>
+      </c>
+      <c r="C216" t="n">
+        <v>23103</v>
+      </c>
+      <c r="D216" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E216" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B217" t="n">
+        <v>499</v>
+      </c>
+      <c r="C217" t="n">
+        <v>23403</v>
+      </c>
+      <c r="D217" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E217" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B218" t="n">
+        <v>499</v>
+      </c>
+      <c r="C218" t="n">
+        <v>23703</v>
+      </c>
+      <c r="D218" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E218" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B219" t="n">
+        <v>499</v>
+      </c>
+      <c r="C219" t="n">
+        <v>24003</v>
+      </c>
+      <c r="D219" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E219" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B220" t="n">
+        <v>499</v>
+      </c>
+      <c r="C220" t="n">
+        <v>24303</v>
+      </c>
+      <c r="D220" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E220" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B221" t="n">
+        <v>499</v>
+      </c>
+      <c r="C221" t="n">
+        <v>24603</v>
+      </c>
+      <c r="D221" t="n">
+        <v>1.602406592770495</v>
+      </c>
+      <c r="E221" t="n">
+        <v>1.602406592770495</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B222" t="n">
+        <v>500</v>
+      </c>
+      <c r="C222" t="n">
+        <v>24904</v>
+      </c>
+      <c r="D222" t="n">
+        <v>1.207386263014368</v>
+      </c>
+      <c r="E222" t="n">
+        <v>1.207386263014368</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B223" t="n">
+        <v>612</v>
+      </c>
+      <c r="C223" t="n">
+        <v>25204</v>
+      </c>
+      <c r="D223" t="n">
+        <v>1.457341647598808</v>
+      </c>
+      <c r="E223" t="n">
+        <v>1.457341647598808</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B224" t="n">
+        <v>729</v>
+      </c>
+      <c r="C224" t="n">
+        <v>25504</v>
+      </c>
+      <c r="D224" t="n">
+        <v>1.715114701608554</v>
+      </c>
+      <c r="E224" t="n">
+        <v>1.715114701608554</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B225" t="n">
+        <v>902</v>
+      </c>
+      <c r="C225" t="n">
+        <v>25804</v>
+      </c>
+      <c r="D225" t="n">
+        <v>2.097997074791735</v>
+      </c>
+      <c r="E225" t="n">
+        <v>2.097997074791735</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B226" t="n">
+        <v>942</v>
+      </c>
+      <c r="C226" t="n">
+        <v>26104</v>
+      </c>
+      <c r="D226" t="n">
+        <v>2.178998637979132</v>
+      </c>
+      <c r="E226" t="n">
+        <v>2.178998637979132</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B227" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C227" t="n">
+        <v>26404</v>
+      </c>
+      <c r="D227" t="n">
+        <v>2.287044881275042</v>
+      </c>
+      <c r="E227" t="n">
+        <v>2.287044881275042</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B228" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C228" t="n">
+        <v>26704</v>
+      </c>
+      <c r="D228" t="n">
+        <v>2.287044881275042</v>
+      </c>
+      <c r="E228" t="n">
+        <v>2.287044881275042</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>45914.27872456019</v>
+      </c>
+      <c r="B229" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C229" t="n">
+        <v>27004</v>
+      </c>
+      <c r="D229" t="n">
+        <v>2.287044881275042</v>
+      </c>
+      <c r="E229" t="n">
+        <v>2.287044881275042</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>45914.27872456511</v>
+      </c>
+      <c r="B230" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C230" t="n">
+        <v>27067</v>
+      </c>
+      <c r="D230" t="n">
+        <v>2.246745437865594</v>
+      </c>
+      <c r="E230" t="n">
+        <v>2.246745437865594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>